<commit_message>
Mark dataset as hypothetical; drop satisfaction
Clarify that the project portfolio is a hypothetical, AI-training dataset and remove the Client Satisfaction column from the workbook and generation script. Updated user-facing text to recommend Copilot / Microsoft Copilot and Cashman AI Portal options, adjusted prompts/hints/systemPrompt to note the dataset is made-up and that satisfaction is not present, and tweaked Excel layout (headers, merges, column widths, notes) accordingly. The generator script now ignores the obsolete satisfaction field (kept in source tuples for diffing), fixes column/index handling and output formatting. Also updates the packaged .xlsx to match these changes.
</commit_message>
<xml_diff>
--- a/public/downloads/cashman-project-portfolio.xlsx
+++ b/public/downloads/cashman-project-portfolio.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -511,20 +511,19 @@
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cashman Companies — Project Portfolio (last 5 years)</t>
+          <t>Cashman Companies — Hypothetical Project Portfolio (training data)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>32 completed (or in-progress) projects across Dredging, Pile Driving, IPC Lydon, and Preload Cryogenics. Use this dataset to ask AI which project type tends to go over budget and why.</t>
+          <t>32 hypothetical projects across Dredging, Pile Driving, IPC Lydon, and Preload Cryogenics. All names, regions, and figures are made up for AI-training use only. Ask AI which project type tends to go over budget and why.</t>
         </is>
       </c>
     </row>
@@ -587,15 +586,10 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Client Satisfaction (1-5)</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -641,15 +635,12 @@
       <c r="K5" s="5" t="n">
         <v>80000</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>5</v>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Bobby M.</t>
+        </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>Bobby M.</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -695,15 +686,12 @@
       <c r="K6" s="8" t="n">
         <v>920000</v>
       </c>
-      <c r="L6" s="9" t="n">
-        <v>4</v>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Bobby M.</t>
+        </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>Bobby M.</t>
-        </is>
-      </c>
-      <c r="N6" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -749,15 +737,12 @@
       <c r="K7" s="5" t="n">
         <v>140000</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>5</v>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Sarah K.</t>
+        </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Sarah K.</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -803,15 +788,12 @@
       <c r="K8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="9" t="n">
-        <v>5</v>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Bobby M.</t>
+        </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>Bobby M.</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -857,15 +839,12 @@
       <c r="K9" s="5" t="n">
         <v>1350000</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>3</v>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Sarah K.</t>
+        </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>Sarah K.</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -911,15 +890,12 @@
       <c r="K10" s="8" t="n">
         <v>280000</v>
       </c>
-      <c r="L10" s="9" t="n">
-        <v>5</v>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Bobby M.</t>
+        </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>Bobby M.</t>
-        </is>
-      </c>
-      <c r="N10" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -965,15 +941,12 @@
       <c r="K11" s="5" t="n">
         <v>55000</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>4</v>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Sarah K.</t>
+        </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>Sarah K.</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1019,15 +992,12 @@
       <c r="K12" s="8" t="n">
         <v>165000</v>
       </c>
-      <c r="L12" s="9" t="n">
-        <v>4</v>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Bobby M.</t>
+        </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>Bobby M.</t>
-        </is>
-      </c>
-      <c r="N12" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1073,15 +1043,12 @@
       <c r="K13" s="5" t="n">
         <v>145000</v>
       </c>
-      <c r="L13" s="6" t="n">
-        <v>4</v>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Mike R.</t>
+        </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>Mike R.</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1127,15 +1094,12 @@
       <c r="K14" s="8" t="n">
         <v>180000</v>
       </c>
-      <c r="L14" s="9" t="n">
-        <v>4</v>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>Mike R.</t>
+        </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>Mike R.</t>
-        </is>
-      </c>
-      <c r="N14" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1181,15 +1145,12 @@
       <c r="K15" s="5" t="n">
         <v>45000</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>5</v>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1235,15 +1196,12 @@
       <c r="K16" s="8" t="n">
         <v>60000</v>
       </c>
-      <c r="L16" s="9" t="n">
-        <v>5</v>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Mike R.</t>
+        </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
-        <is>
-          <t>Mike R.</t>
-        </is>
-      </c>
-      <c r="N16" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1289,15 +1247,12 @@
       <c r="K17" s="5" t="n">
         <v>680000</v>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>4</v>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1343,15 +1298,12 @@
       <c r="K18" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="L18" s="9" t="n">
-        <v>5</v>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>Mike R.</t>
+        </is>
       </c>
       <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>Mike R.</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1397,15 +1349,12 @@
       <c r="K19" s="5" t="n">
         <v>520000</v>
       </c>
-      <c r="L19" s="6" t="n">
-        <v>4</v>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1451,15 +1400,12 @@
       <c r="K20" s="8" t="n">
         <v>42000</v>
       </c>
-      <c r="L20" s="9" t="n">
-        <v>5</v>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Mike R.</t>
+        </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>Mike R.</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1505,15 +1451,12 @@
       <c r="K21" s="5" t="n">
         <v>860000</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>3</v>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Peter S.</t>
+        </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
-        <is>
-          <t>Peter S.</t>
-        </is>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1559,15 +1502,12 @@
       <c r="K22" s="8" t="n">
         <v>1350000</v>
       </c>
-      <c r="L22" s="9" t="n">
-        <v>2</v>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>Peter S.</t>
+        </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>Peter S.</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1613,15 +1553,12 @@
       <c r="K23" s="5" t="n">
         <v>280000</v>
       </c>
-      <c r="L23" s="6" t="n">
-        <v>4</v>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1667,15 +1604,12 @@
       <c r="K24" s="8" t="n">
         <v>75000</v>
       </c>
-      <c r="L24" s="9" t="n">
-        <v>4</v>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N24" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1721,15 +1655,12 @@
       <c r="K25" s="5" t="n">
         <v>720000</v>
       </c>
-      <c r="L25" s="6" t="n">
-        <v>3</v>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Peter S.</t>
+        </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
-        <is>
-          <t>Peter S.</t>
-        </is>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1775,15 +1706,12 @@
       <c r="K26" s="8" t="n">
         <v>55000</v>
       </c>
-      <c r="L26" s="9" t="n">
-        <v>5</v>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N26" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1829,15 +1757,12 @@
       <c r="K27" s="5" t="n">
         <v>1450000</v>
       </c>
-      <c r="L27" s="6" t="n">
-        <v>3</v>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Peter S.</t>
+        </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>Peter S.</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1883,15 +1808,12 @@
       <c r="K28" s="8" t="n">
         <v>3900000</v>
       </c>
-      <c r="L28" s="9" t="n">
-        <v>2</v>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>Peter S.</t>
+        </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
-        <is>
-          <t>Peter S.</t>
-        </is>
-      </c>
-      <c r="N28" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1937,15 +1859,12 @@
       <c r="K29" s="5" t="n">
         <v>380000</v>
       </c>
-      <c r="L29" s="6" t="n">
-        <v>5</v>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1991,15 +1910,12 @@
       <c r="K30" s="8" t="n">
         <v>7400000</v>
       </c>
-      <c r="L30" s="9" t="n">
-        <v>2</v>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N30" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2045,15 +1961,12 @@
       <c r="K31" s="5" t="n">
         <v>12900000</v>
       </c>
-      <c r="L31" s="6" t="n">
-        <v>2</v>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2099,15 +2012,12 @@
       <c r="K32" s="8" t="n">
         <v>1500000</v>
       </c>
-      <c r="L32" s="9" t="n">
-        <v>4</v>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N32" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2153,15 +2063,12 @@
       <c r="K33" s="5" t="n">
         <v>600000</v>
       </c>
-      <c r="L33" s="6" t="n">
-        <v>5</v>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2207,15 +2114,12 @@
       <c r="K34" s="8" t="n">
         <v>3800000</v>
       </c>
-      <c r="L34" s="9" t="n">
-        <v>2</v>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N34" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2261,15 +2165,12 @@
       <c r="K35" s="5" t="n">
         <v>5500000</v>
       </c>
-      <c r="L35" s="6" t="n">
-        <v>3</v>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Karen H.</t>
+        </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
-        <is>
-          <t>Karen H.</t>
-        </is>
-      </c>
-      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2315,15 +2216,12 @@
       <c r="K36" s="8" t="n">
         <v>15200000</v>
       </c>
-      <c r="L36" s="9" t="n">
-        <v>2</v>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>Wes T.</t>
+        </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
-        <is>
-          <t>Wes T.</t>
-        </is>
-      </c>
-      <c r="N36" s="7" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -2339,21 +2237,21 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>• Cost Variance = Final Cost − Contract Value (positive = over budget)</t>
+          <t>• All project names, regions, and figures in this workbook are HYPOTHETICAL and exist for AI-training purposes only.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>• Schedule Variance = Actual Duration − Planned Duration (positive = late)</t>
+          <t>• Cost Variance = Final Cost − Contract Value (positive = over budget)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>• Client Satisfaction is on a 1 (worst) to 5 (best) scale, captured at project closeout</t>
+          <t>• Schedule Variance = Actual Duration − Planned Duration (positive = late)</t>
         </is>
       </c>
     </row>
@@ -2364,23 +2262,15 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>• All figures are hypothetical and for training only</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A40:N40"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A43:N43"/>
-    <mergeCell ref="A41:N41"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="A44:N44"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A40:M40"/>
+    <mergeCell ref="A39:M39"/>
+    <mergeCell ref="A43:M43"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A42:M42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>